<commit_message>
Update clinical_trial_data.xlsx with new test sheets
</commit_message>
<xml_diff>
--- a/example_data/clinical_trial_data.xlsx
+++ b/example_data/clinical_trial_data.xlsx
@@ -6,7 +6,9 @@
     <sheet name="Patients" sheetId="1" r:id="rId1"/>
     <sheet name="Samples" sheetId="2" r:id="rId2"/>
     <sheet name="Treatments" sheetId="3" r:id="rId3"/>
-    <sheet name="Empty_Sheet" sheetId="4" r:id="rId4"/>
+    <sheet name="Patients_Append" sheetId="4" r:id="rId4"/>
+    <sheet name="Patients_Upsert" sheetId="5" r:id="rId5"/>
+    <sheet name="Empty_Sheet" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -724,6 +726,147 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>patient_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>age</v>
+      </c>
+      <c r="C1" t="str">
+        <v>gender</v>
+      </c>
+      <c r="D1" t="str">
+        <v>diagnosis_date</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>P006</v>
+      </c>
+      <c r="B2">
+        <v>60</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2023-06-01</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Alive</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>P007</v>
+      </c>
+      <c r="B3">
+        <v>41</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Female</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2023-06-15</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Alive</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>patient_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>age</v>
+      </c>
+      <c r="C1" t="str">
+        <v>gender</v>
+      </c>
+      <c r="D1" t="str">
+        <v>diagnosis_date</v>
+      </c>
+      <c r="E1" t="str">
+        <v>status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>P001</v>
+      </c>
+      <c r="B2">
+        <v>45</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2023-01-15</v>
+      </c>
+      <c r="E2" t="str">
+        <v>In Remission</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>P002</v>
+      </c>
+      <c r="B3">
+        <v>32</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Female</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2023-02-20</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Deceased</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>P008</v>
+      </c>
+      <c r="B4">
+        <v>22</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2023-07-20</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Alive</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetData/>
   <ignoredErrors>

</xml_diff>